<commit_message>
IT move to 2025
</commit_message>
<xml_diff>
--- a/InputData/plcy-schd/IT/Initial Time.xlsx
+++ b/InputData/plcy-schd/IT/Initial Time.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\plcy-schd\IT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OliviaAshmoore\Documents\Github Repos\eps-us\InputData\plcy-schd\IT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AA8C60E-CEBA-45F4-A6A5-57AAB35EBDA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECD54F93-26AC-4324-B576-68E813F28100}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -451,14 +451,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -466,52 +466,52 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
@@ -519,12 +519,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
@@ -532,12 +532,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>20</v>
       </c>
@@ -554,19 +554,19 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2">
-        <v>2024</v>
+        <v>2025</v>
       </c>
     </row>
   </sheetData>

</xml_diff>